<commit_message>
Add dojo system, 2R1201ev, 2RDEVIL event, and stats recalculation
</commit_message>
<xml_diff>
--- a/files/CHR/talk_プロセル.xlsx
+++ b/files/CHR/talk_プロセル.xlsx
@@ -495,7 +495,7 @@
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>ノア</t>
+          <t>プロセル</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>指、5本……うん、当然だな</t>
+          <t>……この指、借り物にしては良く出来ている</t>
         </is>
       </c>
     </row>
@@ -515,7 +515,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>この魔導書の重さ、体の使い方を変えたら気にならなくなった</t>
+          <t>得物の重さなど、我には関係のない話だ</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>腹が減った……ボクの分の食料も、ちゃんと確保しておかないと</t>
+          <t>腹が減る、か……人の子の感覚とは、面白いものだな</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>これだけ植物があって食える実がひとつもないなんて、道理に合わないな</t>
+          <t>緑ばかりで実らぬとは……この地もまだ、地獄に劣るな</t>
         </is>
       </c>
     </row>
@@ -545,7 +545,7 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>甘いもの……糖分は、頭を使う時こそ必要だ</t>
+          <t>温かい飲み物……人の子はそんなものを恋しがるのか</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>声は出る。……問題ない</t>
+          <t>……この声も、借り物か。まあ、悪くはない</t>
         </is>
       </c>
     </row>
@@ -565,7 +565,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>……今のは風か。……音の出所くらい、すぐわかる</t>
+          <t>風、か。……我を脅かすには、あまりに軽い</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>独り言というより、考えを声に出してるだけだ。そのほうが整理しやすい</t>
+          <t>独り言というより……お前たちに聞かせているのだがな</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>12月でこの暖かさ……理屈に合わないな、これは</t>
+          <t>この寒さのなさ、……地獄の方がまだ、温もりがある</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>靴擦れしないな、これ……体、なにか変わってる気がする</t>
+          <t>傷ひとつつかぬ足か。……人の子にしては上出来だ</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>今日、何日だっけ……誰かが数えてるなら、任せておくか</t>
+          <t>日付など、我には意味のない単位だ</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>さっきの……あまり嫌な感触じゃなかった。……それが、少し引っかかる</t>
+          <t>……あの手応え、悪くなかった。お前、少しずつ強くなっているな</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>疲れた……けど、休むよりまだ動けそうだ</t>
+          <t>疲れ、か。……その感覚も、久しく忘れていたものだ</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>蝶……いや、落ち葉か。見間違えた</t>
+          <t>蝶……ではなく、ただの葉か。つまらん</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>飛行機雲……あれ、ずっと止まってるな</t>
+          <t>あの雲、止まったままだな。……この世界そのものが、時を止めているようだ</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>今の音……なんだろうな。……ちょっと、様子見だ</t>
+          <t>今の音……。ふん、警戒するがいい。それでこそ、お前だ</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>影、一個多い気がした……気のせいにしとくか</t>
+          <t>影がひとつ多い、か。……我のことは、勘定に入れなくてよい</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>猫かと思ったら根っこか……紛らわしいな</t>
+          <t>猫でも、根でも……どちらでも我には同じことだ</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>風、なんかお出汁の匂いする……腹が減ってるだけだろうな</t>
+          <t>出汁の匂い、か。人の子の腹は、実に忙しない</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>焼き芋屋さんの音、した気がした……そんな平和なもの、あるわけないのに</t>
+          <t>……焼き芋、とやらの音。この地に、まだそんな平穏が残っているとはな</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>1、2、3、4……よし、5本ある</t>
+          <t>1、2、3、4、5……我にとっては、数など飾りに過ぎぬが</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>一人で生き延びるのと、みんなでいるのと……どう考えても後者の方がマシだ。合流して正解だったな</t>
+          <t>あの魔導書の主、少し気になってはいるのだがな……連れの小娘の加護が、鬱陶しいほど効く</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>ボクの魔導書、まだ使ったことない術式があるんだよな……試せる時が来たら、試してみたい</t>
+          <t>お前が強くなるほど、我が故郷へ還る道も開ける……励むといい</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>自販機、空か……まあ、そんなもんだろうな</t>
+          <t>自販機、空か。……この文明の残骸、もう少し役に立てばよいものを</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>静かだな……こういうとこの方が、ものを考えやすい</t>
+          <t>誰もおらぬ、か。……我にとっては、これが常の景色だ</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>血じゃなくて樹液、だよな……そういうことにしておく</t>
+          <t>血ではなく樹液、か。……この世界、随分と生ぬるい嘘をつく</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>電波塔としては世界一の高さだったはずだ……この崩れ方だと、相当頑丈な作りだったんだろうな</t>
+          <t>電波塔、とやら……人の子は、天に近づきたがる生き物だな</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>新幹線の駅だったはずだ……交通の要所だった場所は、後で拠点にするなら悪くないかもな</t>
+          <t>駅、か……人が群れ、運ばれる場所。家畜と大差ない</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>京橋……あんまり詳しくないな、ここは</t>
+          <t>知らぬ地名だ。興味もない</t>
         </is>
       </c>
     </row>
@@ -803,7 +803,7 @@
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>日本一人が集まる駅だったはずだ……これだけ人がいた場所なら、物資も残ってるかもしれない</t>
+          <t>人が最も集まったという場所か。……今はこの静けさとは、皮肉なものだ</t>
         </is>
       </c>
     </row>
@@ -815,7 +815,7 @@
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>江戸城か……昔の防御の作り方、今のボクらにも参考になりそうだな</t>
+          <t>城、か。……人の子の権威の象徴など、我には滑稽に映る</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>正門ってことは、動線がちゃんと考えられてる作りなんだろうな</t>
+          <t>門、か。……この程度の結界、我には無いも同然だがな</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>赤レンガの駅舎……有名だったはずなのに、見る影もないな</t>
+          <t>駅舎、赤き煉瓦……美しいと思ったこともあったが、今は瓦礫だ</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>コリアンタウンだったはずだ……今は関係ないけど</t>
+          <t>異国の食が集まる地、か。……我には無縁の話だ</t>
         </is>
       </c>
     </row>
@@ -863,7 +863,7 @@
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>オフィス街か……人が多かった場所なら、非常食とか残ってそうだな</t>
+          <t>働く者たちの巣、か。……人の子は、実によく働く生き物だ</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>あんまり知らないな、ここは</t>
+          <t>知らぬ地だ</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>渋滞してそうな通りだな、昔は</t>
+          <t>かつては車が連なっていたのだろうな。今は、風だけが通る</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>カメラ屋さん多そうな通りだな……使えるもの、残ってるかもな</t>
+          <t>光学の道具を扱う店、か……人の子の技術も、時に侮れぬ</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>6車線……こんな道路、和歌山にはなかったな</t>
+          <t>これほどの道幅、人の子にしては大胆な発想だ</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>博物館とか動物園があったはずだ……資料が残ってたら、貴重かもな</t>
+          <t>古き寺、か。……祈りとは、我らにとっても餌になる</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>電気街だったはずだ……部品の宝庫だったんだろうな、昔は</t>
+          <t>電気の街、か。……人の子の欲は、実に多彩だ</t>
         </is>
       </c>
     </row>
@@ -947,7 +947,7 @@
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>ドーム球場か……あの構造、拠点にするにはよさそうだけど</t>
+          <t>球戯の殿堂、か。……あの歓声は、もう聞けぬのだろうな</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>300階建てって……よくそんなの建てたな、昔の人</t>
+          <t>三百層とは……人の子は、天まで届く塔を好むな</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>333メートル、だったはずだ……今はもう、意味ないけど</t>
+          <t>電波塔、赤きもの……人の子の見栄というものよ</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>テーマパークか……今は関係ないな</t>
+          <t>夢を見せる場所、だったか。……この地には、もう似合わぬな</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>独特な匂いする街だな……理由は考えたくないな</t>
+          <t>この匂い……人の子の弱さが、染み付いた地だな</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>シーサー……魔除けだったはずだ</t>
+          <t>魔除けの像、か。……その程度で我らを退けられると思うなよ</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>観覧車と水族館……水があるなら、水源として使えるかもな</t>
+          <t>回る車と、魚の檻か……人の子の娯楽とは、つくづく奇妙だ</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>イベントやってた痕跡だな……いつ頃かは分からないけど</t>
+          <t>祭りの跡、か。……賑わいの残り香すら、もう腐っている</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>神社か……建物、意外としっかり残ってるな</t>
+          <t>神を祀る場所、か……その神は、今どこにいる</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>道路に電車……変わった街だったんだな、ここ</t>
+          <t>道に電車、とは……人の子の工夫、嫌いではない</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>あんまり知らないな、ここは</t>
+          <t>知らぬ地だ、興味もない</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>モノレールだったはずだ……乗ったことないけど</t>
+          <t>軌条の乗り物、か……我には縁のない話だ</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>展示会場だったはずだ……広いし、拠点にするには悪くなさそうだな</t>
+          <t>物を並べ、競う場、か……人の子の見栄の張り合いは飽きぬな</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>あの見た目……UFOってわけじゃないだろうけど、何のためにあんな形にしたんだか</t>
+          <t>あの形……人の子か、それとも別の何かの仕業か。判じかねる</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>山が見える……あっちの方が、標高高そうだな</t>
+          <t>山、か。……あの向こうに、まだ何か生きているのだろうか</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>電車……山手線かな。動いてたら助かったのに</t>
+          <t>電車……動かぬ鉄の亡骸だな</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>大きい通りだったんだろうな</t>
+          <t>大きな道だな……かつては、さぞ賑わっていたのだろう</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>ビル群見える……あっちから来たんだったな、覚えとこう</t>
+          <t>ビル群、か……お前たちが来た方角、覚えておくといい</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>潮の匂い……海、近いのかもな</t>
+          <t>潮の匂い……海が近いな</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>高速道路の下か……日陰、休むにはちょうどいいかもな</t>
+          <t>高速の下、か……身を隠すには悪くない</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>埋め立て地か……地面、大丈夫なんだろうか</t>
+          <t>埋め立ての地、か……遠くに、まだ何か残っているようだな</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>来た……大丈夫、対処できる</t>
+          <t>来たか……よかろう、その力、見せてみよ</t>
         </is>
       </c>
     </row>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>なんか嫌な予感……来るぞ</t>
+          <t>嫌な気配だ……ふん、退屈しのぎにはなる</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>この気配……前にもあったな</t>
+          <t>この気配、覚えがあるな</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>よし、来た……落ち着いていこう</t>
+          <t>来たか……存分にやるがいい</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>見つかったか……仕方ない、やるか</t>
+          <t>気づかれたか……面倒だが、仕方あるまい</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>猫じゃなかったな、残念</t>
+          <t>猫かと思えば、違ったか。……つまらぬ</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>囲まれてるな……各個撃破の方が早い</t>
+          <t>囲まれているな……我なら、まとめて葬るがな</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>不意打ちか……でも、対応できる範囲だ</t>
+          <t>ふん、驚いたか。……まだまだ、お前は青いな</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>よし、やろう</t>
+          <t>行け</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>エンカウントか……想定の範囲内だな</t>
+          <t>エンカウント、か……励むがいい</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>待て、まだ準備できてない</t>
+          <t>まだ支度が済んでおらぬようだな</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>あんまりゆっくりしてられないか</t>
+          <t>悠長にはしていられぬか</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>これは……ちょっと厄介そうだな</t>
+          <t>これは……少々、骨が折れそうだな</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>片付けよう</t>
+          <t>さっさと片付けよ</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>……面倒だな</t>
+          <t>……面倒な</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>待て、まだ食べ終わってない</t>
+          <t>まだ食しておる最中だぞ、待て</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>日が暮れるな……早いな</t>
+          <t>日が沈むか……早いものだ</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>もうこんな時間か</t>
+          <t>もうそのような刻限か</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>星、見えてきたな……観測にはいい条件だ</t>
+          <t>星が見えてきたな……地獄からも、同じ星は見えるのだろうか</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>デネブ、ベガ、アルタイル……夏の大三角形だったはずだけど、今の季節には合わないな</t>
+          <t>あの星々の並び……人の子は、勝手に名をつけるものだな</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>飯の時間か……腹減った</t>
+          <t>食の刻限か。……お前たちの腹は、実に忙しない</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>夜が明けたか……よし、生きてる</t>
+          <t>夜が明けたか……よくぞ、生き延びたものだ</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>……おはよう</t>
+          <t>……ふん、おはよう</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>明るいな……よかった</t>
+          <t>明るいな。……悪くはない</t>
         </is>
       </c>
     </row>
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>目が覚めても状況変わらないか……まあ、当然だな</t>
+          <t>目覚めても、この悪夢は続くか……お前も、大概運がないな</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>腹減った……朝飯、なんかあるといいけど</t>
+          <t>腹が減った、か……その感覚、お前から少し移ったかもしれぬな</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>よし、今日の動き方、考えよう</t>
+          <t>よし、今日も励むがいい</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>夜中の地響き……何だったんだろうな、あれ</t>
+          <t>夜半の地響き、か……何かが、また目覚めたのかもしれぬ</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>食料、本当に何もないな……予想はしてたけど</t>
+          <t>何も残っておらぬか。……人の子とは、つくづく脆いものよ</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1547,7 @@
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>もっと計画的に食べればよかったな</t>
+          <t>もう少し、計画的であればよかったものを</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>暗いな……何も見えない</t>
+          <t>闇など、我にはただの景色だ</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>化け物の気配、さっきからずっとするな……消える気配ないな</t>
+          <t>化け物の気配、絶えぬな……この地、随分と賑やかだ</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>もう、すぐそこまで来てるな</t>
+          <t>すぐそこまで来ているな……面白い</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>あちこち崩れて……もう長くもたないな、ここ</t>
+          <t>崩れゆくか……この地も、そう長くはあるまい</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>仕方ない、行くか</t>
+          <t>よかろう、行くとしよう</t>
         </is>
       </c>
     </row>

</xml_diff>